<commit_message>
terminando el modulo de importacion de datos
</commit_message>
<xml_diff>
--- a/app/fixtures/Libro1.xlsx
+++ b/app/fixtures/Libro1.xlsx
@@ -3,17 +3,106 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11985"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Ventas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
+  </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+  <si>
+    <t>Fecha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Producto / Servicio</t>
+  </si>
+  <si>
+    <t>Categoría</t>
+  </si>
+  <si>
+    <t>Cantidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precio Unitario ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Café americano</t>
+  </si>
+  <si>
+    <t>Cafés</t>
+  </si>
+  <si>
+    <t>2.50</t>
+  </si>
+  <si>
+    <t>25.00</t>
+  </si>
+  <si>
+    <t>Desayuno</t>
+  </si>
+  <si>
+    <t>Servicios</t>
+  </si>
+  <si>
+    <t>6.00</t>
+  </si>
+  <si>
+    <t>30.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Combo desayuno</t>
+  </si>
+  <si>
+    <t>Combos</t>
+  </si>
+  <si>
+    <t>5.50</t>
+  </si>
+  <si>
+    <t>44.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jugo natural</t>
+  </si>
+  <si>
+    <t>Jugos</t>
+  </si>
+  <si>
+    <t>2.75</t>
+  </si>
+  <si>
+    <t>27.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Combo merienda</t>
+  </si>
+  <si>
+    <t>Promociones</t>
+  </si>
+  <si>
+    <t>4.00</t>
+  </si>
+  <si>
+    <t>24.00</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <sz val="11.000000"/>
@@ -32,17 +121,20 @@
   </fills>
   <borders count="1">
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -387,74 +479,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface="Arial"/>
         <a:cs typeface="Arial"/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface="Arial"/>
         <a:cs typeface="Arial"/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -462,7 +494,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -488,7 +520,7 @@
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -565,7 +597,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -601,7 +633,138 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="20.8515625"/>
+    <col customWidth="1" min="3" max="3" width="15.8515625"/>
+    <col customWidth="1" min="7" max="7" width="29.8515625"/>
+    <col customWidth="1" min="8" max="8" width="20.57421875"/>
+  </cols>
+  <sheetData>
+    <row r="3" ht="14.25">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" ht="14.25">
+      <c r="A4" s="1">
+        <v>46266</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" ht="14.25">
+      <c r="A5" s="1">
+        <v>46267</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5">
+        <v>5</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" ht="14.25">
+      <c r="A6" s="1">
+        <v>46268</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6">
+        <v>8</v>
+      </c>
+      <c r="E6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" ht="14.25">
+      <c r="A7" s="1">
+        <v>46271</v>
+      </c>
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7">
+        <v>10</v>
+      </c>
+      <c r="E7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" ht="14.25">
+      <c r="A8" s="1">
+        <v>46274</v>
+      </c>
+      <c r="B8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8">
+        <v>6</v>
+      </c>
+      <c r="E8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>